<commit_message>
Implementa automacao completa com SQLite, Pandas e FastAPI
</commit_message>
<xml_diff>
--- a/relatorio.xlsx
+++ b/relatorio.xlsx
@@ -415,353 +415,178 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>data</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>produto</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>produto</t>
+          <t>cliente</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>cliente</t>
+          <t>cidade</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>cidade</t>
+          <t>quantidade</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>quantidade</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
           <t>valor_unitario</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Notebook</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Empresa A</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>São Paulo</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F2" t="n">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Mouse</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Empresa B</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>10</v>
+      </c>
+      <c r="F3" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Monitor</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Empresa C</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Teclado</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Empresa D</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Curitiba</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F5" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Notebook</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Empresa E</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>São Paulo</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Notebook</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Empresa A</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>São Paulo</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G2" t="n">
-        <v>3500</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Mouse</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Empresa B</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Rio de Janeiro</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>10</v>
-      </c>
-      <c r="G3" t="n">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2026-06-02</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Monitor</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Empresa C</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Belo Horizonte</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>3</v>
-      </c>
-      <c r="G4" t="n">
-        <v>1200</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2026-06-02</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Teclado</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Empresa D</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Curitiba</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>5</v>
-      </c>
-      <c r="G5" t="n">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>2026-06-03</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Notebook</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Empresa E</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>São Paulo</t>
-        </is>
-      </c>
       <c r="F6" t="n">
-        <v>1</v>
-      </c>
-      <c r="G6" t="n">
-        <v>3500</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Notebook</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Empresa A</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>São Paulo</t>
-        </is>
-      </c>
-      <c r="F7" t="n">
-        <v>2</v>
-      </c>
-      <c r="G7" t="n">
-        <v>3500</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Mouse</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Empresa B</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Rio de Janeiro</t>
-        </is>
-      </c>
-      <c r="F8" t="n">
-        <v>10</v>
-      </c>
-      <c r="G8" t="n">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>2026-06-02</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Monitor</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Empresa C</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Belo Horizonte</t>
-        </is>
-      </c>
-      <c r="F9" t="n">
-        <v>3</v>
-      </c>
-      <c r="G9" t="n">
-        <v>1200</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>2026-06-02</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Teclado</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Empresa D</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Curitiba</t>
-        </is>
-      </c>
-      <c r="F10" t="n">
-        <v>5</v>
-      </c>
-      <c r="G10" t="n">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>2026-06-03</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Notebook</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Empresa E</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>São Paulo</t>
-        </is>
-      </c>
-      <c r="F11" t="n">
-        <v>1</v>
-      </c>
-      <c r="G11" t="n">
         <v>3500</v>
       </c>
     </row>
@@ -798,7 +623,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>21000</v>
+        <v>10500</v>
       </c>
     </row>
     <row r="3">
@@ -808,7 +633,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>7200</v>
+        <v>3600</v>
       </c>
     </row>
     <row r="4">
@@ -818,7 +643,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1600</v>
+        <v>800</v>
       </c>
     </row>
     <row r="5">
@@ -828,7 +653,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1500</v>
+        <v>750</v>
       </c>
     </row>
   </sheetData>
@@ -864,7 +689,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>21000</v>
+        <v>10500</v>
       </c>
     </row>
     <row r="3">
@@ -874,7 +699,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>7200</v>
+        <v>3600</v>
       </c>
     </row>
     <row r="4">
@@ -884,7 +709,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1600</v>
+        <v>800</v>
       </c>
     </row>
     <row r="5">
@@ -894,7 +719,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1500</v>
+        <v>750</v>
       </c>
     </row>
   </sheetData>

</xml_diff>